<commit_message>
progress: 70 village workbooks (sivaramans-llin 2026-10-10T19:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitoornatham_13.414965_80.056991.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chitoornatham_13.414965_80.056991.xlsx
@@ -1118,6 +1118,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1125,6 +1130,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 3C, 3D, 3E1, 3E2, 3F1, 3F2, 3G, 3H, 3I, 3J, 4, 5, 6, 7A, 7B, 8A, 8B, 8C, 8D, 8E, 8F, 8G, 9</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1132,6 +1142,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1139,6 +1154,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1146,6 +1166,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 19C, 19D, 2, 20A, 20B, 20C, 21, 22, 23, 24, 25, 26, 27, 28, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1153,6 +1178,11 @@
           <t>654</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1160,6 +1190,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1167,6 +1202,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1174,6 +1214,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1181,6 +1226,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 5C, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1188,6 +1238,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 3, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1195,6 +1250,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21A, 21B, 21C, 22, 23, 24A, 24B, 24C, 24D, 25, 26, 27, 28, 29, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 37, 38, 39, 4, 40, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1202,6 +1262,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1209,6 +1274,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1216,6 +1286,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1223,6 +1298,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B1A, 18B1B, 18B1C1, 18B1C2, 18B2A, 18B2B1, 18B2B2, 18C1A, 18C1B, 18C2, 18C3, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1230,6 +1310,11 @@
           <t>749</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1237,6 +1322,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1244,6 +1334,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1251,6 +1346,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1258,6 +1358,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1265,6 +1370,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 18C, 19A, 19B, 19C, 2, 20A, 20B, 20C, 20D, 20E, 20F, 20G, 21A, 21B, 22A, 22B, 22C, 22D, 23, 24, 25A, 25B, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1272,6 +1382,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4A, 4B, 5, 6, 7A, 7B, 7C, 7D1, 7D2, 7D3, 7E, 7F1, 7F2, 7F3, 7G, 7H, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1279,6 +1394,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1286,6 +1406,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1293,6 +1418,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1300,6 +1430,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1307,6 +1442,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1314,6 +1454,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14, 1A, 1B, 1C1, 1C2, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1321,6 +1466,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27A, 27B, 28A, 28B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1328,6 +1478,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1C1, 1C2, 1D1, 1D2, 1E, 2, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1335,6 +1490,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15A, 15B, 15C, 16, 17A, 17B, 18, 19A, 19B, 19C, 1A, 1B, 1C, 2, 20, 21, 3, 4A, 4B, 4C, 5A1, 5A2, 5B, 6A, 6B, 6C, 6D, 7A, 7B, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1342,6 +1502,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 21A, 21B, 21C, 22, 23, 24, 25, 26, 27, 28A, 28B, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1349,6 +1514,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1356,6 +1526,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16A, 16B, 17, 18, 19A, 19B, 20, 2A, 2B, 2C, 2D, 3A, 3B, 4, 5A, 5B, 6, 7, 8A, 8B1, 8B2, 8B3, 8B4, 8B5, 8B6, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1363,6 +1538,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2A1A, 2A1B, 2A2, 2A3A, 2A3B, 2A4, 2A5, 2A6, 2A7, 2A8A, 2A8B, 2A9, 2B, 3, 4A, 4B1, 4B2, 4B3, 4B4, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1370,6 +1550,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1377,6 +1562,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1384,6 +1574,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1391,6 +1586,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1398,6 +1598,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1405,6 +1610,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11A3, 12, 13, 14, 15A, 15B, 15C, 16A, 16B, 17, 18, 19A, 19B, 2, 20, 21A, 21B, 22, 23, 3, 4, 5A, 5B, 6, 7A, 7B, 7C1, 7C2, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1412,11 +1622,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16A, 16B, 16C, 17A, 17B, 18A, 18B, 19, 20A, 20B, 21, 22, 23A1, 23A2, 23B1, 23B2, 24, 25, 26, 27, 2A, 2B, 2C, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4A, 4B, 4C, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>